<commit_message>
Version 1.0; add example strategies, enums, unit-comp, compiler
</commit_message>
<xml_diff>
--- a/data/build-orders/ff-islands-galley.xlsx
+++ b/data/build-orders/ff-islands-galley.xlsx
@@ -1,24 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/58a644f44110df98/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/58a644f44110df98/Repos/aoe2-ai-strategy-builder/data/build-orders/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="708" documentId="8_{F4964CE7-B815-4871-98B8-16CE05AE9DEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4A1D619D-3446-4887-92A8-9C3347B61753}"/>
+  <xr:revisionPtr revIDLastSave="712" documentId="8_{F4964CE7-B815-4871-98B8-16CE05AE9DEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1EB3E468-20DC-4BD6-812F-982250DC1668}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{F8A9DD4B-4318-4779-A8E0-EFA21C27FDD3}"/>
+    <workbookView xWindow="2280" yWindow="2280" windowWidth="19200" windowHeight="11170" firstSheet="1" activeTab="3" xr2:uid="{F8A9DD4B-4318-4779-A8E0-EFA21C27FDD3}"/>
   </bookViews>
   <sheets>
     <sheet name="build-order" sheetId="1" r:id="rId1"/>
     <sheet name="vill-numbers" sheetId="2" r:id="rId2"/>
-    <sheet name="allowed-civs" sheetId="3" r:id="rId3"/>
-    <sheet name="allowed-positions" sheetId="6" r:id="rId4"/>
-    <sheet name="allowed-maps" sheetId="4" r:id="rId5"/>
-    <sheet name="options" sheetId="5" r:id="rId6"/>
+    <sheet name="civs" sheetId="3" r:id="rId3"/>
+    <sheet name="positions" sheetId="6" r:id="rId4"/>
+    <sheet name="map-style" sheetId="4" r:id="rId5"/>
+    <sheet name="map-type" sheetId="7" r:id="rId6"/>
+    <sheet name="options" sheetId="5" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="136">
   <si>
     <t>item</t>
   </si>
@@ -178,9 +179,6 @@
     <t>italian</t>
   </si>
   <si>
-    <t>indian</t>
-  </si>
-  <si>
     <t>hindustanis</t>
   </si>
   <si>
@@ -289,9 +287,6 @@
     <t>value</t>
   </si>
   <si>
-    <t>Av</t>
-  </si>
-  <si>
     <t>ri-bodkin-arrow</t>
   </si>
   <si>
@@ -325,6 +320,9 @@
     <t>5 villager-wood, dock</t>
   </si>
   <si>
+    <t>fire-galley</t>
+  </si>
+  <si>
     <t>blacksmith, 10 class-warship</t>
   </si>
   <si>
@@ -340,7 +338,31 @@
     <t>2 dock, gold-mining-camp, 6 class-warship</t>
   </si>
   <si>
-    <t>galley</t>
+    <t>U</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>macedonians</t>
+  </si>
+  <si>
+    <t>thracians</t>
+  </si>
+  <si>
+    <t>puru</t>
+  </si>
+  <si>
+    <t>muisca</t>
+  </si>
+  <si>
+    <t>mapuche</t>
+  </si>
+  <si>
+    <t>tupi</t>
+  </si>
+  <si>
+    <t>maybe</t>
   </si>
   <si>
     <t>style-arabia</t>
@@ -361,12 +383,24 @@
     <t>style-random</t>
   </si>
   <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>If True</t>
+  </si>
+  <si>
+    <t>If False</t>
+  </si>
+  <si>
     <t>map-multipleTCs</t>
   </si>
   <si>
     <t>map-startingWalls</t>
   </si>
   <si>
+    <t>no</t>
+  </si>
+  <si>
     <t>map-nomadStart</t>
   </si>
   <si>
@@ -394,52 +428,28 @@
     <t>map-migrationStart</t>
   </si>
   <si>
-    <t>map-wallable</t>
-  </si>
-  <si>
-    <t>land-unit-percent</t>
-  </si>
-  <si>
-    <t>allow defensive spearmen</t>
-  </si>
-  <si>
-    <t>allow defensive monks</t>
-  </si>
-  <si>
-    <t>allow defensive siege</t>
-  </si>
-  <si>
-    <t>counter-unit-factor</t>
-  </si>
-  <si>
-    <t>agressivness-factor</t>
-  </si>
-  <si>
-    <t>micro-level</t>
-  </si>
-  <si>
-    <t>economy-speed</t>
-  </si>
-  <si>
-    <t>population-percent</t>
-  </si>
-  <si>
-    <t>macedonians</t>
-  </si>
-  <si>
-    <t>thracians</t>
-  </si>
-  <si>
-    <t>puru</t>
-  </si>
-  <si>
-    <t>muisca</t>
-  </si>
-  <si>
-    <t>mapuche</t>
-  </si>
-  <si>
-    <t>tupi</t>
+    <t>map-wallable-med</t>
+  </si>
+  <si>
+    <t>drop-res</t>
+  </si>
+  <si>
+    <t>2 drop-res</t>
+  </si>
+  <si>
+    <t>map-wallable-easy</t>
+  </si>
+  <si>
+    <t>map-wallable-hard</t>
+  </si>
+  <si>
+    <t>Defence::KILL_RAM_DIST</t>
+  </si>
+  <si>
+    <t>Defence::KILL_RAM_AVOID_ENEMY_DIST</t>
+  </si>
+  <si>
+    <t>Defence::KILL_RAM_VILLAGER_DIST</t>
   </si>
 </sst>
 </file>
@@ -606,11 +616,11 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -627,6 +637,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -951,7 +965,7 @@
   <cols>
     <col min="1" max="1" width="17.453125" style="1" customWidth="1"/>
     <col min="2" max="4" width="5.453125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="35.7265625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="29" style="1" customWidth="1"/>
     <col min="6" max="6" width="17.26953125" style="1" customWidth="1"/>
     <col min="7" max="7" width="82.26953125" customWidth="1"/>
   </cols>
@@ -996,7 +1010,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B3" s="2">
         <v>4</v>
@@ -1008,13 +1022,13 @@
         <v>0</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="G3" s="1"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B4" s="2">
         <v>7</v>
@@ -1026,13 +1040,13 @@
         <v>100</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G4" s="1"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B5" s="2">
         <v>9</v>
@@ -1044,13 +1058,13 @@
         <v>110</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G5" s="1"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="B6" s="2">
         <v>-1</v>
@@ -1065,7 +1079,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B7" s="2">
         <v>2</v>
@@ -1077,13 +1091,13 @@
         <v>0</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="G7" s="1"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B8" s="2">
         <v>1</v>
@@ -1095,13 +1109,13 @@
         <v>100</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G8" s="1"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B9" s="2">
         <v>1</v>
@@ -1113,12 +1127,15 @@
         <v>0</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="9" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B10" s="2">
         <v>2</v>
@@ -1130,13 +1147,16 @@
         <v>20</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>130</v>
       </c>
       <c r="G10" s="1"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B11" s="2">
         <v>3</v>
@@ -1148,7 +1168,7 @@
         <v>100</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
@@ -1165,13 +1185,16 @@
         <v>100</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>129</v>
       </c>
       <c r="G12" s="1"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="9" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B13" s="2">
         <v>1</v>
@@ -1184,6 +1207,9 @@
       </c>
       <c r="E13" s="1" t="s">
         <v>5</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>129</v>
       </c>
       <c r="G13" s="1"/>
     </row>
@@ -1221,6 +1247,9 @@
       <c r="E15" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="F15" s="1" t="s">
+        <v>129</v>
+      </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="10" t="s">
@@ -1235,8 +1264,11 @@
       <c r="D16" s="2">
         <v>90</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F16" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="10" t="s">
         <v>8</v>
       </c>
@@ -1249,8 +1281,11 @@
       <c r="D17" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F17" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="10" t="s">
         <v>10</v>
       </c>
@@ -1264,9 +1299,9 @@
         <v>110</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="10" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B19" s="2">
         <v>1</v>
@@ -1277,8 +1312,11 @@
       <c r="D19" s="2">
         <v>170</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F19" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="11" t="s">
         <v>9</v>
       </c>
@@ -1292,12 +1330,15 @@
         <v>100</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+        <v>87</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" s="11" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B21" s="2">
         <v>1</v>
@@ -1309,12 +1350,12 @@
         <v>190</v>
       </c>
       <c r="E21" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A22" s="11" t="s">
         <v>89</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A22" s="11" t="s">
-        <v>91</v>
       </c>
       <c r="B22" s="2">
         <v>1</v>
@@ -1326,28 +1367,28 @@
         <v>180</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B29"/>
       <c r="C29"/>
       <c r="D29"/>
       <c r="E29"/>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B30"/>
       <c r="C30"/>
       <c r="D30"/>
       <c r="E30"/>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B31"/>
       <c r="C31"/>
       <c r="D31"/>
       <c r="E31"/>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B32"/>
       <c r="C32"/>
       <c r="D32"/>
@@ -1441,9 +1482,7 @@
   <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="2.81640625" customWidth="1"/>
-    <col min="2" max="2" width="3.6328125" customWidth="1"/>
-    <col min="3" max="7" width="2.81640625" customWidth="1"/>
+    <col min="1" max="7" width="3.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -1466,7 +1505,7 @@
         <v>18</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>82</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
@@ -1798,499 +1837,490 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E235E04A-9A12-4DB7-91ED-5AE9B1A234A7}">
-  <dimension ref="A1:B61"/>
+  <dimension ref="A1:B60"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.54296875" customWidth="1"/>
-    <col min="2" max="2" width="7.26953125" style="14" customWidth="1"/>
+    <col min="1" max="1" width="10.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="14">
-        <v>1</v>
+      <c r="B1" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="14">
-        <v>1</v>
+      <c r="B2" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="14">
-        <v>1</v>
+      <c r="B3" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B4" s="14">
-        <v>1</v>
+      <c r="B4" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="B5" s="14">
-        <v>1</v>
+      <c r="B5" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B6" s="14">
-        <v>1</v>
+      <c r="B6" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="14">
-        <v>1</v>
+      <c r="B7" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="14">
-        <v>1</v>
+      <c r="B8" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="14">
-        <v>1</v>
+      <c r="B9" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="14">
-        <v>1</v>
+      <c r="B10" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B11" s="14">
-        <v>1</v>
+      <c r="B11" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="14">
-        <v>1</v>
+      <c r="B12" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="B13" s="14">
-        <v>1</v>
+      <c r="B13" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B14" s="14">
-        <v>1</v>
+      <c r="B14" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="B15" s="14">
-        <v>1</v>
+      <c r="B15" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="B16" s="14">
-        <v>1</v>
+      <c r="B16" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B17" s="14">
-        <v>1</v>
+      <c r="B17" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="B18" s="14">
-        <v>1</v>
+      <c r="B18" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B19" s="14">
-        <v>1</v>
+      <c r="B19" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="B20" s="14">
-        <v>1</v>
+      <c r="B20" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B21" s="14">
-        <v>1</v>
+      <c r="B21" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="B22" s="14">
-        <v>1</v>
+      <c r="B22" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="B23" s="14">
-        <v>1</v>
+      <c r="B23" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="B24" s="14">
-        <v>1</v>
+      <c r="B24" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B25" s="14">
-        <v>1</v>
+      <c r="B25" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B26" s="14">
-        <v>1</v>
+      <c r="B26" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="B27" s="14">
-        <v>1</v>
+      <c r="B27" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B28" s="14">
-        <v>1</v>
+      <c r="B28" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="B29" s="14">
-        <v>1</v>
+      <c r="B29" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="B30" s="14">
-        <v>1</v>
+      <c r="B30" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="B31" s="14">
-        <v>1</v>
+      <c r="B31" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="B32" s="14">
-        <v>1</v>
+      <c r="B32" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="B33" s="14">
-        <v>1</v>
+      <c r="B33" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B34" s="14">
-        <v>1</v>
+      <c r="B34" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="B35" s="14">
-        <v>1</v>
+      <c r="B35" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B36" s="14">
-        <v>1</v>
+      <c r="B36" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="B37" s="14">
-        <v>1</v>
+      <c r="B37" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B38" s="14">
-        <v>1</v>
+      <c r="B38" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="B39" s="14">
-        <v>1</v>
+      <c r="B39" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="B40" s="14">
-        <v>1</v>
+      <c r="B40" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="B41" s="14">
-        <v>1</v>
+      <c r="B41" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="B42" s="14">
-        <v>1</v>
+      <c r="B42" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="B43" s="14">
-        <v>1</v>
+      <c r="B43" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="B44" s="14">
-        <v>1</v>
+      <c r="B44" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A45" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="B45" s="14">
-        <v>1</v>
+      <c r="B45" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="B46" s="14">
-        <v>1</v>
+      <c r="B46" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A47" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="B47" s="14">
-        <v>1</v>
+      <c r="B47" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="B48" s="14">
-        <v>1</v>
+      <c r="B48" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="B49" s="14">
-        <v>1</v>
+      <c r="B49" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="B50" s="14">
-        <v>1</v>
+      <c r="B50" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="B51" s="14">
-        <v>1</v>
+      <c r="B51" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="B52" s="14">
-        <v>1</v>
+      <c r="B52" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A53" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B53" s="14">
-        <v>1</v>
+      <c r="B53" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A54" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="B54" s="14">
-        <v>1</v>
+      <c r="B54" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="B55" s="14">
-        <v>1</v>
+        <v>100</v>
+      </c>
+      <c r="B55" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A56" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="B56" s="14">
-        <v>1</v>
+        <v>101</v>
+      </c>
+      <c r="B56" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A57" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="B57" s="14">
-        <v>1</v>
+        <v>102</v>
+      </c>
+      <c r="B57" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A58" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="B58" s="14">
-        <v>1</v>
+        <v>103</v>
+      </c>
+      <c r="B58" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A59" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="B59" s="14">
-        <v>1</v>
+        <v>104</v>
+      </c>
+      <c r="B59" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A60" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="B60" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A61" s="7" t="s">
-        <v>132</v>
-      </c>
-      <c r="B61" s="14">
-        <v>1</v>
+        <v>105</v>
+      </c>
+      <c r="B60" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -2304,39 +2334,38 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.7265625" customWidth="1"/>
-    <col min="2" max="2" width="5.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>22</v>
       </c>
-      <c r="B1">
-        <v>1</v>
+      <c r="B1" s="7" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>20</v>
       </c>
-      <c r="B2">
-        <v>1</v>
+      <c r="B2" s="7" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>21</v>
       </c>
-      <c r="B3">
-        <v>1</v>
+      <c r="B3" s="7" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>25</v>
       </c>
-      <c r="B4">
-        <v>1</v>
+      <c r="B4" s="7" t="s">
+        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -2346,119 +2375,58 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19248840-518E-4289-A595-9956D1669EEB}">
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.6328125" customWidth="1"/>
-    <col min="2" max="2" width="5.7265625" customWidth="1"/>
+    <col min="1" max="1" width="17.26953125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>100</v>
-      </c>
-      <c r="B1">
-        <v>0</v>
+        <v>107</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>101</v>
-      </c>
-      <c r="B2">
-        <v>0</v>
+        <v>108</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>102</v>
-      </c>
-      <c r="B3">
-        <v>1</v>
+        <v>109</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>103</v>
-      </c>
-      <c r="B4">
-        <v>0</v>
+        <v>110</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>104</v>
-      </c>
-      <c r="B5">
-        <v>0</v>
+        <v>111</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>105</v>
-      </c>
-      <c r="B6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
+        <v>112</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>106</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>117</v>
       </c>
     </row>
   </sheetData>
@@ -2467,92 +2435,221 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11ECD89E-83A2-4D13-B683-1AE2D2F40C42}">
-  <dimension ref="A1:B10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B59BECCD-901C-4F40-BFF1-8CB413FF8A29}">
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.6328125" customWidth="1"/>
-    <col min="2" max="2" width="6.1796875" style="14" customWidth="1"/>
+    <col min="1" max="1" width="17.7265625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>114</v>
+      </c>
+      <c r="C1" s="16" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>120</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>121</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>122</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>123</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>124</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>125</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>126</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>127</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>131</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>128</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>132</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>99</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11ECD89E-83A2-4D13-B683-1AE2D2F40C42}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="35.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" s="15" t="s">
+      <c r="A1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B1" t="s">
         <v>80</v>
-      </c>
-      <c r="B1" s="16" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>118</v>
-      </c>
-      <c r="B2" s="14">
-        <v>0</v>
+        <v>133</v>
+      </c>
+      <c r="B2">
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>119</v>
-      </c>
-      <c r="B3" s="14">
-        <v>1</v>
+        <v>134</v>
+      </c>
+      <c r="B3">
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>120</v>
-      </c>
-      <c r="B4" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>121</v>
-      </c>
-      <c r="B5" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>122</v>
-      </c>
-      <c r="B6" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>123</v>
-      </c>
-      <c r="B7" s="14">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>124</v>
-      </c>
-      <c r="B8" s="14">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>125</v>
-      </c>
-      <c r="B9" s="14">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>126</v>
-      </c>
-      <c r="B10" s="14">
-        <v>100</v>
+        <v>135</v>
+      </c>
+      <c r="B4">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>